<commit_message>
Enhancement: Customizable columns, improved sorting, and UI polish
</commit_message>
<xml_diff>
--- a/Newdata/入庫TECO狀態.XLSX
+++ b/Newdata/入庫TECO狀態.XLSX
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1456" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1456" uniqueCount="343">
   <si>
     <t>ZP02</t>
   </si>
@@ -379,7 +379,7 @@
     <t>200006606</t>
   </si>
   <si>
-    <t>REL  MSPT PRC  MANC SETC</t>
+    <t>REL  MSPT PRC  MANC RMWB SETC</t>
   </si>
   <si>
     <t>200006618</t>
@@ -713,9 +713,6 @@
   </si>
   <si>
     <t>HEP機頭G8K,011194_780,55A18,C</t>
-  </si>
-  <si>
-    <t>REL  MSPT PRC  MANC RMWB SETC</t>
   </si>
   <si>
     <t>200006704</t>
@@ -1170,52 +1167,52 @@
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>330</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>342</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -3447,7 +3444,7 @@
         <v>46169</v>
       </c>
       <c r="J46" t="s">
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="K46" t="s">
         <v>5</v>
@@ -3497,7 +3494,7 @@
         <v>46169</v>
       </c>
       <c r="J47" t="s">
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="K47" t="s">
         <v>5</v>
@@ -6247,7 +6244,7 @@
         <v>46190</v>
       </c>
       <c r="J102" t="s">
-        <v>234</v>
+        <v>122</v>
       </c>
       <c r="K102" t="s">
         <v>5</v>
@@ -6273,7 +6270,7 @@
         <v>0</v>
       </c>
       <c r="B103" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C103" s="2">
         <v>1</v>
@@ -6297,7 +6294,7 @@
         <v>46190</v>
       </c>
       <c r="J103" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="K103" t="s">
         <v>5</v>
@@ -6323,19 +6320,19 @@
         <v>0</v>
       </c>
       <c r="B104" t="s">
+        <v>236</v>
+      </c>
+      <c r="C104" s="2">
+        <v>1</v>
+      </c>
+      <c r="D104" s="2">
+        <v>0</v>
+      </c>
+      <c r="E104" t="s">
         <v>237</v>
       </c>
-      <c r="C104" s="2">
-        <v>1</v>
-      </c>
-      <c r="D104" s="2">
-        <v>0</v>
-      </c>
-      <c r="E104" t="s">
+      <c r="F104" t="s">
         <v>238</v>
-      </c>
-      <c r="F104" t="s">
-        <v>239</v>
       </c>
       <c r="G104" s="3">
         <v>46140</v>
@@ -6373,7 +6370,7 @@
         <v>0</v>
       </c>
       <c r="B105" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C105" s="2">
         <v>1</v>
@@ -6382,10 +6379,10 @@
         <v>0</v>
       </c>
       <c r="E105" t="s">
+        <v>237</v>
+      </c>
+      <c r="F105" t="s">
         <v>238</v>
-      </c>
-      <c r="F105" t="s">
-        <v>239</v>
       </c>
       <c r="G105" s="3">
         <v>46140</v>
@@ -6397,7 +6394,7 @@
         <v>46182</v>
       </c>
       <c r="J105" t="s">
-        <v>234</v>
+        <v>122</v>
       </c>
       <c r="K105" t="s">
         <v>5</v>
@@ -6423,19 +6420,19 @@
         <v>0</v>
       </c>
       <c r="B106" t="s">
+        <v>240</v>
+      </c>
+      <c r="C106" s="2">
+        <v>1</v>
+      </c>
+      <c r="D106" s="2">
+        <v>0</v>
+      </c>
+      <c r="E106" t="s">
         <v>241</v>
       </c>
-      <c r="C106" s="2">
-        <v>1</v>
-      </c>
-      <c r="D106" s="2">
-        <v>0</v>
-      </c>
-      <c r="E106" t="s">
+      <c r="F106" t="s">
         <v>242</v>
-      </c>
-      <c r="F106" t="s">
-        <v>243</v>
       </c>
       <c r="G106" s="3">
         <v>46140</v>
@@ -6473,19 +6470,19 @@
         <v>0</v>
       </c>
       <c r="B107" t="s">
+        <v>243</v>
+      </c>
+      <c r="C107" s="2">
+        <v>1</v>
+      </c>
+      <c r="D107" s="2">
+        <v>0</v>
+      </c>
+      <c r="E107" t="s">
         <v>244</v>
       </c>
-      <c r="C107" s="2">
-        <v>1</v>
-      </c>
-      <c r="D107" s="2">
-        <v>0</v>
-      </c>
-      <c r="E107" t="s">
+      <c r="F107" t="s">
         <v>245</v>
-      </c>
-      <c r="F107" t="s">
-        <v>246</v>
       </c>
       <c r="G107" s="3">
         <v>46142</v>
@@ -6523,7 +6520,7 @@
         <v>0</v>
       </c>
       <c r="B108" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C108" s="2">
         <v>1</v>
@@ -6532,10 +6529,10 @@
         <v>0</v>
       </c>
       <c r="E108" t="s">
+        <v>244</v>
+      </c>
+      <c r="F108" t="s">
         <v>245</v>
-      </c>
-      <c r="F108" t="s">
-        <v>246</v>
       </c>
       <c r="G108" s="3">
         <v>46142</v>
@@ -6573,7 +6570,7 @@
         <v>0</v>
       </c>
       <c r="B109" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C109" s="2">
         <v>1</v>
@@ -6582,10 +6579,10 @@
         <v>0</v>
       </c>
       <c r="E109" t="s">
+        <v>244</v>
+      </c>
+      <c r="F109" t="s">
         <v>245</v>
-      </c>
-      <c r="F109" t="s">
-        <v>246</v>
       </c>
       <c r="G109" s="3">
         <v>46142</v>
@@ -6623,7 +6620,7 @@
         <v>0</v>
       </c>
       <c r="B110" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C110" s="2">
         <v>1</v>
@@ -6632,10 +6629,10 @@
         <v>0</v>
       </c>
       <c r="E110" t="s">
+        <v>244</v>
+      </c>
+      <c r="F110" t="s">
         <v>245</v>
-      </c>
-      <c r="F110" t="s">
-        <v>246</v>
       </c>
       <c r="G110" s="3">
         <v>46142</v>
@@ -6673,7 +6670,7 @@
         <v>0</v>
       </c>
       <c r="B111" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C111" s="2">
         <v>1</v>
@@ -6682,10 +6679,10 @@
         <v>0</v>
       </c>
       <c r="E111" t="s">
+        <v>244</v>
+      </c>
+      <c r="F111" t="s">
         <v>245</v>
-      </c>
-      <c r="F111" t="s">
-        <v>246</v>
       </c>
       <c r="G111" s="3">
         <v>46142</v>
@@ -6723,7 +6720,7 @@
         <v>0</v>
       </c>
       <c r="B112" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C112" s="2">
         <v>1</v>
@@ -6732,10 +6729,10 @@
         <v>0</v>
       </c>
       <c r="E112" t="s">
+        <v>244</v>
+      </c>
+      <c r="F112" t="s">
         <v>245</v>
-      </c>
-      <c r="F112" t="s">
-        <v>246</v>
       </c>
       <c r="G112" s="3">
         <v>46142</v>
@@ -6773,7 +6770,7 @@
         <v>0</v>
       </c>
       <c r="B113" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C113" s="2">
         <v>1</v>
@@ -6797,7 +6794,7 @@
         <v>46160</v>
       </c>
       <c r="J113" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="K113" t="s">
         <v>5</v>
@@ -6823,7 +6820,7 @@
         <v>0</v>
       </c>
       <c r="B114" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C114" s="2">
         <v>1</v>
@@ -6847,7 +6844,7 @@
         <v>46162</v>
       </c>
       <c r="J114" t="s">
-        <v>234</v>
+        <v>122</v>
       </c>
       <c r="K114" t="s">
         <v>5</v>
@@ -6873,7 +6870,7 @@
         <v>0</v>
       </c>
       <c r="B115" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C115" s="2">
         <v>1</v>
@@ -6897,7 +6894,7 @@
         <v>46162</v>
       </c>
       <c r="J115" t="s">
-        <v>234</v>
+        <v>122</v>
       </c>
       <c r="K115" t="s">
         <v>5</v>
@@ -6923,7 +6920,7 @@
         <v>0</v>
       </c>
       <c r="B116" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C116" s="2">
         <v>1</v>
@@ -6973,7 +6970,7 @@
         <v>0</v>
       </c>
       <c r="B117" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C117" s="2">
         <v>1</v>
@@ -7023,7 +7020,7 @@
         <v>0</v>
       </c>
       <c r="B118" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C118" s="2">
         <v>1</v>
@@ -7073,19 +7070,19 @@
         <v>0</v>
       </c>
       <c r="B119" t="s">
+        <v>257</v>
+      </c>
+      <c r="C119" s="2">
+        <v>1</v>
+      </c>
+      <c r="D119" s="2">
+        <v>0</v>
+      </c>
+      <c r="E119" t="s">
         <v>258</v>
       </c>
-      <c r="C119" s="2">
-        <v>1</v>
-      </c>
-      <c r="D119" s="2">
-        <v>0</v>
-      </c>
-      <c r="E119" t="s">
+      <c r="F119" t="s">
         <v>259</v>
-      </c>
-      <c r="F119" t="s">
-        <v>260</v>
       </c>
       <c r="G119" s="3">
         <v>46148</v>
@@ -7123,19 +7120,19 @@
         <v>0</v>
       </c>
       <c r="B120" t="s">
+        <v>260</v>
+      </c>
+      <c r="C120" s="2">
+        <v>1</v>
+      </c>
+      <c r="D120" s="2">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
         <v>261</v>
       </c>
-      <c r="C120" s="2">
-        <v>1</v>
-      </c>
-      <c r="D120" s="2">
-        <v>0</v>
-      </c>
-      <c r="E120" t="s">
+      <c r="F120" t="s">
         <v>262</v>
-      </c>
-      <c r="F120" t="s">
-        <v>263</v>
       </c>
       <c r="G120" s="3">
         <v>46148</v>
@@ -7173,19 +7170,19 @@
         <v>0</v>
       </c>
       <c r="B121" t="s">
+        <v>263</v>
+      </c>
+      <c r="C121" s="2">
+        <v>1</v>
+      </c>
+      <c r="D121" s="2">
+        <v>0</v>
+      </c>
+      <c r="E121" t="s">
         <v>264</v>
       </c>
-      <c r="C121" s="2">
-        <v>1</v>
-      </c>
-      <c r="D121" s="2">
-        <v>0</v>
-      </c>
-      <c r="E121" t="s">
+      <c r="F121" t="s">
         <v>265</v>
-      </c>
-      <c r="F121" t="s">
-        <v>266</v>
       </c>
       <c r="G121" s="3">
         <v>46148</v>
@@ -7197,7 +7194,7 @@
         <v>46162</v>
       </c>
       <c r="J121" t="s">
-        <v>234</v>
+        <v>122</v>
       </c>
       <c r="K121" t="s">
         <v>5</v>
@@ -7223,19 +7220,19 @@
         <v>0</v>
       </c>
       <c r="B122" t="s">
+        <v>266</v>
+      </c>
+      <c r="C122" s="2">
+        <v>1</v>
+      </c>
+      <c r="D122" s="2">
+        <v>0</v>
+      </c>
+      <c r="E122" t="s">
         <v>267</v>
       </c>
-      <c r="C122" s="2">
-        <v>1</v>
-      </c>
-      <c r="D122" s="2">
-        <v>0</v>
-      </c>
-      <c r="E122" t="s">
+      <c r="F122" t="s">
         <v>268</v>
-      </c>
-      <c r="F122" t="s">
-        <v>269</v>
       </c>
       <c r="G122" s="3">
         <v>46148</v>
@@ -7273,19 +7270,19 @@
         <v>0</v>
       </c>
       <c r="B123" t="s">
+        <v>269</v>
+      </c>
+      <c r="C123" s="2">
+        <v>1</v>
+      </c>
+      <c r="D123" s="2">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
         <v>270</v>
       </c>
-      <c r="C123" s="2">
-        <v>1</v>
-      </c>
-      <c r="D123" s="2">
-        <v>0</v>
-      </c>
-      <c r="E123" t="s">
+      <c r="F123" t="s">
         <v>271</v>
-      </c>
-      <c r="F123" t="s">
-        <v>272</v>
       </c>
       <c r="G123" s="3">
         <v>46148</v>
@@ -7323,19 +7320,19 @@
         <v>0</v>
       </c>
       <c r="B124" t="s">
+        <v>272</v>
+      </c>
+      <c r="C124" s="2">
+        <v>1</v>
+      </c>
+      <c r="D124" s="2">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
         <v>273</v>
       </c>
-      <c r="C124" s="2">
-        <v>1</v>
-      </c>
-      <c r="D124" s="2">
-        <v>0</v>
-      </c>
-      <c r="E124" t="s">
+      <c r="F124" t="s">
         <v>274</v>
-      </c>
-      <c r="F124" t="s">
-        <v>275</v>
       </c>
       <c r="G124" s="3">
         <v>46148</v>
@@ -7373,19 +7370,19 @@
         <v>0</v>
       </c>
       <c r="B125" t="s">
+        <v>275</v>
+      </c>
+      <c r="C125" s="2">
+        <v>1</v>
+      </c>
+      <c r="D125" s="2">
+        <v>0</v>
+      </c>
+      <c r="E125" t="s">
         <v>276</v>
       </c>
-      <c r="C125" s="2">
-        <v>1</v>
-      </c>
-      <c r="D125" s="2">
-        <v>0</v>
-      </c>
-      <c r="E125" t="s">
+      <c r="F125" t="s">
         <v>277</v>
-      </c>
-      <c r="F125" t="s">
-        <v>278</v>
       </c>
       <c r="G125" s="3">
         <v>46148</v>
@@ -7423,19 +7420,19 @@
         <v>0</v>
       </c>
       <c r="B126" t="s">
+        <v>278</v>
+      </c>
+      <c r="C126" s="2">
+        <v>1</v>
+      </c>
+      <c r="D126" s="2">
+        <v>0</v>
+      </c>
+      <c r="E126" t="s">
         <v>279</v>
       </c>
-      <c r="C126" s="2">
-        <v>1</v>
-      </c>
-      <c r="D126" s="2">
-        <v>0</v>
-      </c>
-      <c r="E126" t="s">
+      <c r="F126" t="s">
         <v>280</v>
-      </c>
-      <c r="F126" t="s">
-        <v>281</v>
       </c>
       <c r="G126" s="3">
         <v>46148</v>
@@ -7473,19 +7470,19 @@
         <v>0</v>
       </c>
       <c r="B127" t="s">
+        <v>281</v>
+      </c>
+      <c r="C127" s="2">
+        <v>1</v>
+      </c>
+      <c r="D127" s="2">
+        <v>0</v>
+      </c>
+      <c r="E127" t="s">
         <v>282</v>
       </c>
-      <c r="C127" s="2">
-        <v>1</v>
-      </c>
-      <c r="D127" s="2">
-        <v>0</v>
-      </c>
-      <c r="E127" t="s">
+      <c r="F127" t="s">
         <v>283</v>
-      </c>
-      <c r="F127" t="s">
-        <v>284</v>
       </c>
       <c r="G127" s="3">
         <v>46148</v>
@@ -7523,19 +7520,19 @@
         <v>0</v>
       </c>
       <c r="B128" t="s">
+        <v>284</v>
+      </c>
+      <c r="C128" s="2">
+        <v>1</v>
+      </c>
+      <c r="D128" s="2">
+        <v>0</v>
+      </c>
+      <c r="E128" t="s">
         <v>285</v>
       </c>
-      <c r="C128" s="2">
-        <v>1</v>
-      </c>
-      <c r="D128" s="2">
-        <v>0</v>
-      </c>
-      <c r="E128" t="s">
+      <c r="F128" t="s">
         <v>286</v>
-      </c>
-      <c r="F128" t="s">
-        <v>287</v>
       </c>
       <c r="G128" s="3">
         <v>46148</v>
@@ -7573,19 +7570,19 @@
         <v>0</v>
       </c>
       <c r="B129" t="s">
+        <v>287</v>
+      </c>
+      <c r="C129" s="2">
+        <v>1</v>
+      </c>
+      <c r="D129" s="2">
+        <v>0</v>
+      </c>
+      <c r="E129" t="s">
         <v>288</v>
       </c>
-      <c r="C129" s="2">
-        <v>1</v>
-      </c>
-      <c r="D129" s="2">
-        <v>0</v>
-      </c>
-      <c r="E129" t="s">
+      <c r="F129" t="s">
         <v>289</v>
-      </c>
-      <c r="F129" t="s">
-        <v>290</v>
       </c>
       <c r="G129" s="3">
         <v>46153</v>
@@ -7597,7 +7594,7 @@
         <v>46202</v>
       </c>
       <c r="J129" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K129" t="s">
         <v>5</v>
@@ -7623,19 +7620,19 @@
         <v>0</v>
       </c>
       <c r="B130" t="s">
+        <v>291</v>
+      </c>
+      <c r="C130" s="2">
+        <v>1</v>
+      </c>
+      <c r="D130" s="2">
+        <v>0</v>
+      </c>
+      <c r="E130" t="s">
         <v>292</v>
       </c>
-      <c r="C130" s="2">
-        <v>1</v>
-      </c>
-      <c r="D130" s="2">
-        <v>0</v>
-      </c>
-      <c r="E130" t="s">
+      <c r="F130" t="s">
         <v>293</v>
-      </c>
-      <c r="F130" t="s">
-        <v>294</v>
       </c>
       <c r="G130" s="3">
         <v>46153</v>
@@ -7673,19 +7670,19 @@
         <v>0</v>
       </c>
       <c r="B131" t="s">
+        <v>294</v>
+      </c>
+      <c r="C131" s="2">
+        <v>1</v>
+      </c>
+      <c r="D131" s="2">
+        <v>0</v>
+      </c>
+      <c r="E131" t="s">
         <v>295</v>
       </c>
-      <c r="C131" s="2">
-        <v>1</v>
-      </c>
-      <c r="D131" s="2">
-        <v>0</v>
-      </c>
-      <c r="E131" t="s">
+      <c r="F131" t="s">
         <v>296</v>
-      </c>
-      <c r="F131" t="s">
-        <v>297</v>
       </c>
       <c r="G131" s="3">
         <v>46153</v>
@@ -7723,19 +7720,19 @@
         <v>0</v>
       </c>
       <c r="B132" t="s">
+        <v>297</v>
+      </c>
+      <c r="C132" s="2">
+        <v>1</v>
+      </c>
+      <c r="D132" s="2">
+        <v>0</v>
+      </c>
+      <c r="E132" t="s">
         <v>298</v>
       </c>
-      <c r="C132" s="2">
-        <v>1</v>
-      </c>
-      <c r="D132" s="2">
-        <v>0</v>
-      </c>
-      <c r="E132" t="s">
+      <c r="F132" t="s">
         <v>299</v>
-      </c>
-      <c r="F132" t="s">
-        <v>300</v>
       </c>
       <c r="G132" s="3">
         <v>46153</v>
@@ -7747,7 +7744,7 @@
         <v>46161</v>
       </c>
       <c r="J132" t="s">
-        <v>234</v>
+        <v>122</v>
       </c>
       <c r="K132" t="s">
         <v>5</v>
@@ -7773,19 +7770,19 @@
         <v>0</v>
       </c>
       <c r="B133" t="s">
+        <v>300</v>
+      </c>
+      <c r="C133" s="2">
+        <v>1</v>
+      </c>
+      <c r="D133" s="2">
+        <v>0</v>
+      </c>
+      <c r="E133" t="s">
         <v>301</v>
       </c>
-      <c r="C133" s="2">
-        <v>1</v>
-      </c>
-      <c r="D133" s="2">
-        <v>0</v>
-      </c>
-      <c r="E133" t="s">
+      <c r="F133" t="s">
         <v>302</v>
-      </c>
-      <c r="F133" t="s">
-        <v>303</v>
       </c>
       <c r="G133" s="3">
         <v>46153</v>
@@ -7797,7 +7794,7 @@
         <v>46156</v>
       </c>
       <c r="J133" t="s">
-        <v>55</v>
+        <v>167</v>
       </c>
       <c r="K133" t="s">
         <v>5</v>
@@ -7823,19 +7820,19 @@
         <v>0</v>
       </c>
       <c r="B134" t="s">
+        <v>303</v>
+      </c>
+      <c r="C134" s="2">
+        <v>1</v>
+      </c>
+      <c r="D134" s="2">
+        <v>0</v>
+      </c>
+      <c r="E134" t="s">
         <v>304</v>
       </c>
-      <c r="C134" s="2">
-        <v>1</v>
-      </c>
-      <c r="D134" s="2">
-        <v>0</v>
-      </c>
-      <c r="E134" t="s">
+      <c r="F134" t="s">
         <v>305</v>
-      </c>
-      <c r="F134" t="s">
-        <v>306</v>
       </c>
       <c r="G134" s="3">
         <v>46154</v>
@@ -7873,19 +7870,19 @@
         <v>0</v>
       </c>
       <c r="B135" t="s">
+        <v>306</v>
+      </c>
+      <c r="C135" s="2">
+        <v>1</v>
+      </c>
+      <c r="D135" s="2">
+        <v>0</v>
+      </c>
+      <c r="E135" t="s">
         <v>307</v>
       </c>
-      <c r="C135" s="2">
-        <v>1</v>
-      </c>
-      <c r="D135" s="2">
-        <v>0</v>
-      </c>
-      <c r="E135" t="s">
+      <c r="F135" t="s">
         <v>308</v>
-      </c>
-      <c r="F135" t="s">
-        <v>309</v>
       </c>
       <c r="G135" s="3">
         <v>46154</v>
@@ -7923,7 +7920,7 @@
         <v>0</v>
       </c>
       <c r="B136" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C136" s="2">
         <v>1</v>
@@ -7973,16 +7970,16 @@
         <v>0</v>
       </c>
       <c r="B137" t="s">
+        <v>310</v>
+      </c>
+      <c r="C137" s="2">
+        <v>1</v>
+      </c>
+      <c r="D137" s="2">
+        <v>0</v>
+      </c>
+      <c r="E137" t="s">
         <v>311</v>
-      </c>
-      <c r="C137" s="2">
-        <v>1</v>
-      </c>
-      <c r="D137" s="2">
-        <v>0</v>
-      </c>
-      <c r="E137" t="s">
-        <v>312</v>
       </c>
       <c r="F137" t="s">
         <v>228</v>
@@ -8023,7 +8020,7 @@
         <v>0</v>
       </c>
       <c r="B138" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C138" s="2">
         <v>1</v>
@@ -8073,7 +8070,7 @@
         <v>0</v>
       </c>
       <c r="B139" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C139" s="2">
         <v>1</v>
@@ -8082,10 +8079,10 @@
         <v>0</v>
       </c>
       <c r="E139" t="s">
+        <v>258</v>
+      </c>
+      <c r="F139" t="s">
         <v>259</v>
-      </c>
-      <c r="F139" t="s">
-        <v>260</v>
       </c>
       <c r="G139" s="3">
         <v>46156</v>
@@ -8123,7 +8120,7 @@
         <v>0</v>
       </c>
       <c r="B140" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C140" s="2">
         <v>1</v>
@@ -8132,10 +8129,10 @@
         <v>0</v>
       </c>
       <c r="E140" t="s">
+        <v>258</v>
+      </c>
+      <c r="F140" t="s">
         <v>259</v>
-      </c>
-      <c r="F140" t="s">
-        <v>260</v>
       </c>
       <c r="G140" s="3">
         <v>46156</v>
@@ -8173,7 +8170,7 @@
         <v>0</v>
       </c>
       <c r="B141" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C141" s="2">
         <v>1</v>
@@ -8197,7 +8194,7 @@
         <v>46168</v>
       </c>
       <c r="J141" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="K141" t="s">
         <v>5</v>
@@ -8223,7 +8220,7 @@
         <v>0</v>
       </c>
       <c r="B142" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C142" s="2">
         <v>1</v>
@@ -8247,7 +8244,7 @@
         <v>46162</v>
       </c>
       <c r="J142" t="s">
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="K142" t="s">
         <v>5</v>
@@ -8270,22 +8267,22 @@
     </row>
     <row r="143" spans="1:16">
       <c r="A143" t="s">
+        <v>318</v>
+      </c>
+      <c r="B143" t="s">
         <v>319</v>
       </c>
-      <c r="B143" t="s">
+      <c r="C143" s="2">
+        <v>1</v>
+      </c>
+      <c r="D143" s="2">
+        <v>0</v>
+      </c>
+      <c r="E143" t="s">
         <v>320</v>
       </c>
-      <c r="C143" s="2">
-        <v>1</v>
-      </c>
-      <c r="D143" s="2">
-        <v>0</v>
-      </c>
-      <c r="E143" t="s">
+      <c r="F143" t="s">
         <v>321</v>
-      </c>
-      <c r="F143" t="s">
-        <v>322</v>
       </c>
       <c r="G143" s="3">
         <v>46043</v>
@@ -8300,7 +8297,7 @@
         <v>31</v>
       </c>
       <c r="K143" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="L143" s="3">
         <v>46043</v>
@@ -8320,22 +8317,22 @@
     </row>
     <row r="144" spans="1:16">
       <c r="A144" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B144" t="s">
+        <v>323</v>
+      </c>
+      <c r="C144" s="2">
+        <v>1</v>
+      </c>
+      <c r="D144" s="2">
+        <v>0</v>
+      </c>
+      <c r="E144" t="s">
         <v>324</v>
       </c>
-      <c r="C144" s="2">
-        <v>1</v>
-      </c>
-      <c r="D144" s="2">
-        <v>0</v>
-      </c>
-      <c r="E144" t="s">
+      <c r="F144" t="s">
         <v>325</v>
-      </c>
-      <c r="F144" t="s">
-        <v>326</v>
       </c>
       <c r="G144" s="3">
         <v>46114</v>
@@ -8350,7 +8347,7 @@
         <v>49</v>
       </c>
       <c r="K144" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="L144" s="3">
         <v>46114</v>
@@ -8370,10 +8367,10 @@
     </row>
     <row r="145" spans="1:16">
       <c r="A145" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B145" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C145" s="2">
         <v>1</v>
@@ -8382,10 +8379,10 @@
         <v>0</v>
       </c>
       <c r="E145" t="s">
+        <v>292</v>
+      </c>
+      <c r="F145" t="s">
         <v>293</v>
-      </c>
-      <c r="F145" t="s">
-        <v>294</v>
       </c>
       <c r="G145" s="3">
         <v>46140</v>
@@ -8400,7 +8397,7 @@
         <v>49</v>
       </c>
       <c r="K145" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="L145" s="3">
         <v>46140</v>

</xml_diff>